<commit_message>
Suggested changes and wording implemented
</commit_message>
<xml_diff>
--- a/docs/assets/capacity_conversion_results_formatted.xlsx
+++ b/docs/assets/capacity_conversion_results_formatted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://csucloudservices-my.sharepoint.com/personal/claire_welsh_mlcsu_nhs_uk/Documents/Documents/Strategy Unit/NHP/Capacity Conversion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{2A620748-7BC9-4AC6-81C4-29DAD87E815D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A7F91AB-3255-4CEF-B59D-FFDE4B5B7FC5}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{2A620748-7BC9-4AC6-81C4-29DAD87E815D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FFF5172-B00F-4068-9951-B78B936D08DE}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2233,8 +2233,7 @@
         <v>125</v>
       </c>
       <c r="B2">
-        <f ca="1">RANDBETWEEN(0,10000)</f>
-        <v>7152</v>
+        <v>2000</v>
       </c>
       <c r="C2" t="s">
         <v>225</v>
@@ -2248,8 +2247,7 @@
         <v>126</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B66" ca="1" si="0">RANDBETWEEN(0,10000)</f>
-        <v>5123</v>
+        <v>2000</v>
       </c>
       <c r="C3" t="s">
         <v>225</v>
@@ -2263,8 +2261,7 @@
         <v>127</v>
       </c>
       <c r="B4">
-        <f t="shared" ca="1" si="0"/>
-        <v>8432</v>
+        <v>2000</v>
       </c>
       <c r="C4" t="s">
         <v>225</v>
@@ -2278,8 +2275,7 @@
         <v>128</v>
       </c>
       <c r="B5">
-        <f t="shared" ca="1" si="0"/>
-        <v>7704</v>
+        <v>2000</v>
       </c>
       <c r="C5" t="s">
         <v>225</v>
@@ -2293,8 +2289,7 @@
         <v>134</v>
       </c>
       <c r="B6">
-        <f t="shared" ca="1" si="0"/>
-        <v>8828</v>
+        <v>2000</v>
       </c>
       <c r="C6" t="s">
         <v>226</v>
@@ -2308,8 +2303,7 @@
         <v>135</v>
       </c>
       <c r="B7">
-        <f t="shared" ca="1" si="0"/>
-        <v>8010</v>
+        <v>2000</v>
       </c>
       <c r="C7" t="s">
         <v>226</v>
@@ -2323,8 +2317,7 @@
         <v>136</v>
       </c>
       <c r="B8">
-        <f t="shared" ca="1" si="0"/>
-        <v>7338</v>
+        <v>2000</v>
       </c>
       <c r="C8" t="s">
         <v>226</v>
@@ -2338,8 +2331,7 @@
         <v>137</v>
       </c>
       <c r="B9">
-        <f t="shared" ca="1" si="0"/>
-        <v>8952</v>
+        <v>2000</v>
       </c>
       <c r="C9" t="s">
         <v>226</v>
@@ -2353,8 +2345,7 @@
         <v>138</v>
       </c>
       <c r="B10">
-        <f t="shared" ca="1" si="0"/>
-        <v>3973</v>
+        <v>2000</v>
       </c>
       <c r="C10" t="s">
         <v>226</v>
@@ -2368,8 +2359,7 @@
         <v>139</v>
       </c>
       <c r="B11">
-        <f t="shared" ca="1" si="0"/>
-        <v>8057</v>
+        <v>2000</v>
       </c>
       <c r="C11" t="s">
         <v>226</v>
@@ -2383,8 +2373,7 @@
         <v>146</v>
       </c>
       <c r="B12">
-        <f t="shared" ca="1" si="0"/>
-        <v>6025</v>
+        <v>2000</v>
       </c>
       <c r="C12" t="s">
         <v>244</v>
@@ -2398,8 +2387,7 @@
         <v>147</v>
       </c>
       <c r="B13">
-        <f t="shared" ca="1" si="0"/>
-        <v>9176</v>
+        <v>2000</v>
       </c>
       <c r="C13" t="s">
         <v>244</v>
@@ -2413,8 +2401,7 @@
         <v>148</v>
       </c>
       <c r="B14">
-        <f t="shared" ca="1" si="0"/>
-        <v>5793</v>
+        <v>2000</v>
       </c>
       <c r="C14" t="s">
         <v>244</v>
@@ -2428,8 +2415,7 @@
         <v>149</v>
       </c>
       <c r="B15">
-        <f t="shared" ca="1" si="0"/>
-        <v>1181</v>
+        <v>2000</v>
       </c>
       <c r="C15" t="s">
         <v>244</v>
@@ -2443,8 +2429,7 @@
         <v>150</v>
       </c>
       <c r="B16">
-        <f t="shared" ca="1" si="0"/>
-        <v>1174</v>
+        <v>2000</v>
       </c>
       <c r="C16" t="s">
         <v>244</v>
@@ -2458,8 +2443,7 @@
         <v>151</v>
       </c>
       <c r="B17">
-        <f t="shared" ca="1" si="0"/>
-        <v>3086</v>
+        <v>2000</v>
       </c>
       <c r="C17" t="s">
         <v>244</v>
@@ -2473,8 +2457,7 @@
         <v>152</v>
       </c>
       <c r="B18">
-        <f t="shared" ca="1" si="0"/>
-        <v>5534</v>
+        <v>2000</v>
       </c>
       <c r="C18" t="s">
         <v>244</v>
@@ -2488,8 +2471,7 @@
         <v>162</v>
       </c>
       <c r="B19">
-        <f t="shared" ca="1" si="0"/>
-        <v>7502</v>
+        <v>2000</v>
       </c>
       <c r="C19" t="s">
         <v>244</v>
@@ -2503,8 +2485,7 @@
         <v>165</v>
       </c>
       <c r="B20">
-        <f t="shared" ca="1" si="0"/>
-        <v>7972</v>
+        <v>2000</v>
       </c>
       <c r="C20" t="s">
         <v>244</v>
@@ -2518,8 +2499,7 @@
         <v>166</v>
       </c>
       <c r="B21">
-        <f t="shared" ca="1" si="0"/>
-        <v>1005</v>
+        <v>2000</v>
       </c>
       <c r="C21" t="s">
         <v>244</v>
@@ -2533,8 +2513,7 @@
         <v>167</v>
       </c>
       <c r="B22">
-        <f t="shared" ca="1" si="0"/>
-        <v>2583</v>
+        <v>2000</v>
       </c>
       <c r="C22" t="s">
         <v>244</v>
@@ -2548,8 +2527,7 @@
         <v>168</v>
       </c>
       <c r="B23">
-        <f t="shared" ca="1" si="0"/>
-        <v>8781</v>
+        <v>2000</v>
       </c>
       <c r="C23" t="s">
         <v>244</v>
@@ -2563,8 +2541,7 @@
         <v>169</v>
       </c>
       <c r="B24">
-        <f t="shared" ca="1" si="0"/>
-        <v>1595</v>
+        <v>2000</v>
       </c>
       <c r="C24" t="s">
         <v>244</v>
@@ -2578,8 +2555,7 @@
         <v>170</v>
       </c>
       <c r="B25">
-        <f t="shared" ca="1" si="0"/>
-        <v>5343</v>
+        <v>2000</v>
       </c>
       <c r="C25" t="s">
         <v>244</v>
@@ -2593,8 +2569,7 @@
         <v>171</v>
       </c>
       <c r="B26">
-        <f t="shared" ca="1" si="0"/>
-        <v>2783</v>
+        <v>2000</v>
       </c>
       <c r="C26" t="s">
         <v>244</v>
@@ -2608,8 +2583,7 @@
         <v>172</v>
       </c>
       <c r="B27">
-        <f t="shared" ca="1" si="0"/>
-        <v>6558</v>
+        <v>2000</v>
       </c>
       <c r="C27" t="s">
         <v>244</v>
@@ -2623,8 +2597,7 @@
         <v>173</v>
       </c>
       <c r="B28">
-        <f t="shared" ca="1" si="0"/>
-        <v>2536</v>
+        <v>2000</v>
       </c>
       <c r="C28" t="s">
         <v>244</v>
@@ -2638,8 +2611,7 @@
         <v>174</v>
       </c>
       <c r="B29">
-        <f t="shared" ca="1" si="0"/>
-        <v>7693</v>
+        <v>2000</v>
       </c>
       <c r="C29" t="s">
         <v>244</v>
@@ -2653,8 +2625,7 @@
         <v>175</v>
       </c>
       <c r="B30">
-        <f t="shared" ca="1" si="0"/>
-        <v>5703</v>
+        <v>2000</v>
       </c>
       <c r="C30" t="s">
         <v>244</v>
@@ -2668,8 +2639,7 @@
         <v>176</v>
       </c>
       <c r="B31">
-        <f t="shared" ca="1" si="0"/>
-        <v>4539</v>
+        <v>2000</v>
       </c>
       <c r="C31" t="s">
         <v>244</v>
@@ -2683,8 +2653,7 @@
         <v>177</v>
       </c>
       <c r="B32">
-        <f t="shared" ca="1" si="0"/>
-        <v>7748</v>
+        <v>2000</v>
       </c>
       <c r="C32" t="s">
         <v>244</v>
@@ -2698,8 +2667,7 @@
         <v>162</v>
       </c>
       <c r="B33">
-        <f t="shared" ca="1" si="0"/>
-        <v>4934</v>
+        <v>2000</v>
       </c>
       <c r="C33" t="s">
         <v>244</v>
@@ -2713,8 +2681,7 @@
         <v>165</v>
       </c>
       <c r="B34">
-        <f t="shared" ca="1" si="0"/>
-        <v>793</v>
+        <v>2000</v>
       </c>
       <c r="C34" t="s">
         <v>244</v>
@@ -2728,8 +2695,7 @@
         <v>166</v>
       </c>
       <c r="B35">
-        <f t="shared" ca="1" si="0"/>
-        <v>3966</v>
+        <v>2000</v>
       </c>
       <c r="C35" t="s">
         <v>244</v>
@@ -2743,8 +2709,7 @@
         <v>167</v>
       </c>
       <c r="B36">
-        <f t="shared" ca="1" si="0"/>
-        <v>5306</v>
+        <v>2000</v>
       </c>
       <c r="C36" t="s">
         <v>244</v>
@@ -2758,8 +2723,7 @@
         <v>168</v>
       </c>
       <c r="B37">
-        <f t="shared" ca="1" si="0"/>
-        <v>6175</v>
+        <v>2000</v>
       </c>
       <c r="C37" t="s">
         <v>244</v>
@@ -2773,8 +2737,7 @@
         <v>169</v>
       </c>
       <c r="B38">
-        <f t="shared" ca="1" si="0"/>
-        <v>6855</v>
+        <v>2000</v>
       </c>
       <c r="C38" t="s">
         <v>244</v>
@@ -2788,8 +2751,7 @@
         <v>170</v>
       </c>
       <c r="B39">
-        <f t="shared" ca="1" si="0"/>
-        <v>722</v>
+        <v>2000</v>
       </c>
       <c r="C39" t="s">
         <v>244</v>
@@ -2803,8 +2765,7 @@
         <v>171</v>
       </c>
       <c r="B40">
-        <f t="shared" ca="1" si="0"/>
-        <v>4557</v>
+        <v>2000</v>
       </c>
       <c r="C40" t="s">
         <v>244</v>
@@ -2818,8 +2779,7 @@
         <v>172</v>
       </c>
       <c r="B41">
-        <f t="shared" ca="1" si="0"/>
-        <v>2912</v>
+        <v>2000</v>
       </c>
       <c r="C41" t="s">
         <v>244</v>
@@ -2833,8 +2793,7 @@
         <v>173</v>
       </c>
       <c r="B42">
-        <f t="shared" ca="1" si="0"/>
-        <v>2733</v>
+        <v>2000</v>
       </c>
       <c r="C42" t="s">
         <v>244</v>
@@ -2848,8 +2807,7 @@
         <v>174</v>
       </c>
       <c r="B43">
-        <f t="shared" ca="1" si="0"/>
-        <v>6781</v>
+        <v>2000</v>
       </c>
       <c r="C43" t="s">
         <v>244</v>
@@ -2863,8 +2821,7 @@
         <v>175</v>
       </c>
       <c r="B44">
-        <f t="shared" ca="1" si="0"/>
-        <v>1153</v>
+        <v>2000</v>
       </c>
       <c r="C44" t="s">
         <v>244</v>
@@ -2878,8 +2835,7 @@
         <v>176</v>
       </c>
       <c r="B45">
-        <f t="shared" ca="1" si="0"/>
-        <v>9453</v>
+        <v>2000</v>
       </c>
       <c r="C45" t="s">
         <v>244</v>
@@ -2893,8 +2849,7 @@
         <v>177</v>
       </c>
       <c r="B46">
-        <f t="shared" ca="1" si="0"/>
-        <v>4311</v>
+        <v>2000</v>
       </c>
       <c r="C46" t="s">
         <v>244</v>
@@ -2908,8 +2863,7 @@
         <v>184</v>
       </c>
       <c r="B47">
-        <f t="shared" ca="1" si="0"/>
-        <v>6222</v>
+        <v>2000</v>
       </c>
       <c r="C47" t="s">
         <v>244</v>
@@ -2923,8 +2877,7 @@
         <v>185</v>
       </c>
       <c r="B48">
-        <f t="shared" ca="1" si="0"/>
-        <v>1429</v>
+        <v>2000</v>
       </c>
       <c r="C48" t="s">
         <v>244</v>
@@ -2938,8 +2891,7 @@
         <v>186</v>
       </c>
       <c r="B49">
-        <f t="shared" ca="1" si="0"/>
-        <v>3119</v>
+        <v>2000</v>
       </c>
       <c r="C49" t="s">
         <v>244</v>
@@ -2953,8 +2905,7 @@
         <v>187</v>
       </c>
       <c r="B50">
-        <f t="shared" ca="1" si="0"/>
-        <v>1024</v>
+        <v>2000</v>
       </c>
       <c r="C50" t="s">
         <v>244</v>
@@ -2968,8 +2919,7 @@
         <v>188</v>
       </c>
       <c r="B51">
-        <f t="shared" ca="1" si="0"/>
-        <v>4669</v>
+        <v>2000</v>
       </c>
       <c r="C51" t="s">
         <v>244</v>
@@ -2983,8 +2933,7 @@
         <v>189</v>
       </c>
       <c r="B52">
-        <f t="shared" ca="1" si="0"/>
-        <v>508</v>
+        <v>2000</v>
       </c>
       <c r="C52" t="s">
         <v>244</v>
@@ -2998,8 +2947,7 @@
         <v>190</v>
       </c>
       <c r="B53">
-        <f t="shared" ca="1" si="0"/>
-        <v>4609</v>
+        <v>2000</v>
       </c>
       <c r="C53" t="s">
         <v>244</v>
@@ -3013,8 +2961,7 @@
         <v>198</v>
       </c>
       <c r="B54">
-        <f t="shared" ca="1" si="0"/>
-        <v>8643</v>
+        <v>2000</v>
       </c>
       <c r="C54" t="s">
         <v>244</v>
@@ -3028,8 +2975,7 @@
         <v>199</v>
       </c>
       <c r="B55">
-        <f t="shared" ca="1" si="0"/>
-        <v>5973</v>
+        <v>2000</v>
       </c>
       <c r="C55" t="s">
         <v>244</v>
@@ -3043,8 +2989,7 @@
         <v>200</v>
       </c>
       <c r="B56">
-        <f t="shared" ca="1" si="0"/>
-        <v>6284</v>
+        <v>2000</v>
       </c>
       <c r="C56" t="s">
         <v>244</v>
@@ -3058,8 +3003,7 @@
         <v>201</v>
       </c>
       <c r="B57">
-        <f t="shared" ca="1" si="0"/>
-        <v>9456</v>
+        <v>2000</v>
       </c>
       <c r="C57" t="s">
         <v>244</v>
@@ -3073,8 +3017,7 @@
         <v>202</v>
       </c>
       <c r="B58">
-        <f t="shared" ca="1" si="0"/>
-        <v>3230</v>
+        <v>2000</v>
       </c>
       <c r="C58" t="s">
         <v>244</v>
@@ -3088,8 +3031,7 @@
         <v>203</v>
       </c>
       <c r="B59">
-        <f t="shared" ca="1" si="0"/>
-        <v>6928</v>
+        <v>2000</v>
       </c>
       <c r="C59" t="s">
         <v>244</v>
@@ -3103,8 +3045,7 @@
         <v>204</v>
       </c>
       <c r="B60">
-        <f t="shared" ca="1" si="0"/>
-        <v>2997</v>
+        <v>2000</v>
       </c>
       <c r="C60" t="s">
         <v>244</v>
@@ -3118,8 +3059,7 @@
         <v>205</v>
       </c>
       <c r="B61">
-        <f t="shared" ca="1" si="0"/>
-        <v>9785</v>
+        <v>2000</v>
       </c>
       <c r="C61" t="s">
         <v>244</v>
@@ -3133,8 +3073,7 @@
         <v>198</v>
       </c>
       <c r="B62">
-        <f t="shared" ca="1" si="0"/>
-        <v>4118</v>
+        <v>2000</v>
       </c>
       <c r="C62" t="s">
         <v>244</v>
@@ -3148,8 +3087,7 @@
         <v>199</v>
       </c>
       <c r="B63">
-        <f t="shared" ca="1" si="0"/>
-        <v>8307</v>
+        <v>2000</v>
       </c>
       <c r="C63" t="s">
         <v>244</v>
@@ -3163,8 +3101,7 @@
         <v>200</v>
       </c>
       <c r="B64">
-        <f t="shared" ca="1" si="0"/>
-        <v>7126</v>
+        <v>2000</v>
       </c>
       <c r="C64" t="s">
         <v>244</v>
@@ -3178,8 +3115,7 @@
         <v>201</v>
       </c>
       <c r="B65">
-        <f t="shared" ca="1" si="0"/>
-        <v>8466</v>
+        <v>2000</v>
       </c>
       <c r="C65" t="s">
         <v>244</v>
@@ -3193,8 +3129,7 @@
         <v>202</v>
       </c>
       <c r="B66">
-        <f t="shared" ca="1" si="0"/>
-        <v>9118</v>
+        <v>2000</v>
       </c>
       <c r="C66" t="s">
         <v>244</v>
@@ -3208,8 +3143,7 @@
         <v>203</v>
       </c>
       <c r="B67">
-        <f t="shared" ref="B67:B69" ca="1" si="1">RANDBETWEEN(0,10000)</f>
-        <v>4423</v>
+        <v>2000</v>
       </c>
       <c r="C67" t="s">
         <v>244</v>
@@ -3223,8 +3157,7 @@
         <v>204</v>
       </c>
       <c r="B68">
-        <f t="shared" ca="1" si="1"/>
-        <v>2172</v>
+        <v>2000</v>
       </c>
       <c r="C68" t="s">
         <v>244</v>
@@ -3238,8 +3171,7 @@
         <v>205</v>
       </c>
       <c r="B69">
-        <f t="shared" ca="1" si="1"/>
-        <v>9180</v>
+        <v>2000</v>
       </c>
       <c r="C69" t="s">
         <v>244</v>
@@ -3287,16 +3219,13 @@
         <v>125</v>
       </c>
       <c r="B2" s="3">
-        <f ca="1">RANDBETWEEN(0,40000)</f>
-        <v>15999</v>
+        <v>10000</v>
       </c>
       <c r="C2" s="3">
-        <f ca="1">RANDBETWEEN(0,40000)</f>
-        <v>33560</v>
+        <v>20000</v>
       </c>
       <c r="D2" s="3">
-        <f ca="1">RANDBETWEEN(0,40000)</f>
-        <v>16687</v>
+        <v>30000</v>
       </c>
       <c r="E2" t="s">
         <v>225</v>
@@ -3310,16 +3239,13 @@
         <v>126</v>
       </c>
       <c r="B3" s="3">
-        <f t="shared" ref="B3:D66" ca="1" si="0">RANDBETWEEN(0,40000)</f>
-        <v>6268</v>
+        <v>10000</v>
       </c>
       <c r="C3" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>13913</v>
+        <v>20000</v>
       </c>
       <c r="D3" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>28467</v>
+        <v>30000</v>
       </c>
       <c r="E3" t="s">
         <v>225</v>
@@ -3333,16 +3259,13 @@
         <v>127</v>
       </c>
       <c r="B4" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39016</v>
+        <v>10000</v>
       </c>
       <c r="C4" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27148</v>
+        <v>20000</v>
       </c>
       <c r="D4" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36312</v>
+        <v>30000</v>
       </c>
       <c r="E4" t="s">
         <v>225</v>
@@ -3356,16 +3279,13 @@
         <v>128</v>
       </c>
       <c r="B5" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>10698</v>
+        <v>10000</v>
       </c>
       <c r="C5" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26244</v>
+        <v>20000</v>
       </c>
       <c r="D5" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8144</v>
+        <v>30000</v>
       </c>
       <c r="E5" t="s">
         <v>225</v>
@@ -3379,16 +3299,13 @@
         <v>134</v>
       </c>
       <c r="B6" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>6437</v>
+        <v>10000</v>
       </c>
       <c r="C6" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>5289</v>
+        <v>20000</v>
       </c>
       <c r="D6" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14499</v>
+        <v>30000</v>
       </c>
       <c r="E6" t="s">
         <v>226</v>
@@ -3402,16 +3319,13 @@
         <v>135</v>
       </c>
       <c r="B7" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14134</v>
+        <v>10000</v>
       </c>
       <c r="C7" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>21886</v>
+        <v>20000</v>
       </c>
       <c r="D7" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>33420</v>
+        <v>30000</v>
       </c>
       <c r="E7" t="s">
         <v>226</v>
@@ -3425,16 +3339,13 @@
         <v>136</v>
       </c>
       <c r="B8" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>22326</v>
+        <v>10000</v>
       </c>
       <c r="C8" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14725</v>
+        <v>20000</v>
       </c>
       <c r="D8" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>2782</v>
+        <v>30000</v>
       </c>
       <c r="E8" t="s">
         <v>226</v>
@@ -3448,16 +3359,13 @@
         <v>137</v>
       </c>
       <c r="B9" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17771</v>
+        <v>10000</v>
       </c>
       <c r="C9" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>25093</v>
+        <v>20000</v>
       </c>
       <c r="D9" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15359</v>
+        <v>30000</v>
       </c>
       <c r="E9" t="s">
         <v>226</v>
@@ -3471,16 +3379,13 @@
         <v>138</v>
       </c>
       <c r="B10" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30554</v>
+        <v>10000</v>
       </c>
       <c r="C10" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>10061</v>
+        <v>20000</v>
       </c>
       <c r="D10" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>23555</v>
+        <v>30000</v>
       </c>
       <c r="E10" t="s">
         <v>226</v>
@@ -3494,16 +3399,13 @@
         <v>139</v>
       </c>
       <c r="B11" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>230</v>
+        <v>10000</v>
       </c>
       <c r="C11" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>38214</v>
+        <v>20000</v>
       </c>
       <c r="D11" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26795</v>
+        <v>30000</v>
       </c>
       <c r="E11" t="s">
         <v>226</v>
@@ -3517,16 +3419,13 @@
         <v>146</v>
       </c>
       <c r="B12" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>5946</v>
+        <v>10000</v>
       </c>
       <c r="C12" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36827</v>
+        <v>20000</v>
       </c>
       <c r="D12" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>22178</v>
+        <v>30000</v>
       </c>
       <c r="E12" t="s">
         <v>244</v>
@@ -3540,16 +3439,13 @@
         <v>147</v>
       </c>
       <c r="B13" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>21673</v>
+        <v>10000</v>
       </c>
       <c r="C13" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>24122</v>
+        <v>20000</v>
       </c>
       <c r="D13" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>29425</v>
+        <v>30000</v>
       </c>
       <c r="E13" t="s">
         <v>244</v>
@@ -3563,16 +3459,13 @@
         <v>148</v>
       </c>
       <c r="B14" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8943</v>
+        <v>10000</v>
       </c>
       <c r="C14" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>21829</v>
+        <v>20000</v>
       </c>
       <c r="D14" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36836</v>
+        <v>30000</v>
       </c>
       <c r="E14" t="s">
         <v>244</v>
@@ -3586,16 +3479,13 @@
         <v>149</v>
       </c>
       <c r="B15" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>38413</v>
+        <v>10000</v>
       </c>
       <c r="C15" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>38218</v>
+        <v>20000</v>
       </c>
       <c r="D15" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30872</v>
+        <v>30000</v>
       </c>
       <c r="E15" t="s">
         <v>244</v>
@@ -3609,16 +3499,13 @@
         <v>150</v>
       </c>
       <c r="B16" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27854</v>
+        <v>10000</v>
       </c>
       <c r="C16" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27288</v>
+        <v>20000</v>
       </c>
       <c r="D16" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>2320</v>
+        <v>30000</v>
       </c>
       <c r="E16" t="s">
         <v>244</v>
@@ -3632,16 +3519,13 @@
         <v>151</v>
       </c>
       <c r="B17" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>34409</v>
+        <v>10000</v>
       </c>
       <c r="C17" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>34748</v>
+        <v>20000</v>
       </c>
       <c r="D17" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>2627</v>
+        <v>30000</v>
       </c>
       <c r="E17" t="s">
         <v>244</v>
@@ -3655,16 +3539,13 @@
         <v>152</v>
       </c>
       <c r="B18" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17931</v>
+        <v>10000</v>
       </c>
       <c r="C18" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32008</v>
+        <v>20000</v>
       </c>
       <c r="D18" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>6366</v>
+        <v>30000</v>
       </c>
       <c r="E18" t="s">
         <v>244</v>
@@ -3678,16 +3559,13 @@
         <v>184</v>
       </c>
       <c r="B19" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>31174</v>
+        <v>10000</v>
       </c>
       <c r="C19" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>23665</v>
+        <v>20000</v>
       </c>
       <c r="D19" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26252</v>
+        <v>30000</v>
       </c>
       <c r="E19" t="s">
         <v>244</v>
@@ -3701,16 +3579,13 @@
         <v>185</v>
       </c>
       <c r="B20" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15380</v>
+        <v>10000</v>
       </c>
       <c r="C20" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32336</v>
+        <v>20000</v>
       </c>
       <c r="D20" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>22060</v>
+        <v>30000</v>
       </c>
       <c r="E20" t="s">
         <v>244</v>
@@ -3724,16 +3599,13 @@
         <v>186</v>
       </c>
       <c r="B21" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35063</v>
+        <v>10000</v>
       </c>
       <c r="C21" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>18186</v>
+        <v>20000</v>
       </c>
       <c r="D21" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>18920</v>
+        <v>30000</v>
       </c>
       <c r="E21" t="s">
         <v>244</v>
@@ -3747,16 +3619,13 @@
         <v>187</v>
       </c>
       <c r="B22" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>9462</v>
+        <v>10000</v>
       </c>
       <c r="C22" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26016</v>
+        <v>20000</v>
       </c>
       <c r="D22" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39415</v>
+        <v>30000</v>
       </c>
       <c r="E22" t="s">
         <v>244</v>
@@ -3770,16 +3639,13 @@
         <v>188</v>
       </c>
       <c r="B23" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>5686</v>
+        <v>10000</v>
       </c>
       <c r="C23" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32293</v>
+        <v>20000</v>
       </c>
       <c r="D23" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>29851</v>
+        <v>30000</v>
       </c>
       <c r="E23" t="s">
         <v>244</v>
@@ -3793,16 +3659,13 @@
         <v>189</v>
       </c>
       <c r="B24" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>25626</v>
+        <v>10000</v>
       </c>
       <c r="C24" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39191</v>
+        <v>20000</v>
       </c>
       <c r="D24" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>13443</v>
+        <v>30000</v>
       </c>
       <c r="E24" t="s">
         <v>244</v>
@@ -3816,16 +3679,13 @@
         <v>190</v>
       </c>
       <c r="B25" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27426</v>
+        <v>10000</v>
       </c>
       <c r="C25" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>16264</v>
+        <v>20000</v>
       </c>
       <c r="D25" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>38318</v>
+        <v>30000</v>
       </c>
       <c r="E25" t="s">
         <v>244</v>
@@ -3839,16 +3699,13 @@
         <v>198</v>
       </c>
       <c r="B26" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8782</v>
+        <v>10000</v>
       </c>
       <c r="C26" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17096</v>
+        <v>20000</v>
       </c>
       <c r="D26" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15992</v>
+        <v>30000</v>
       </c>
       <c r="E26" t="s">
         <v>244</v>
@@ -3862,16 +3719,13 @@
         <v>199</v>
       </c>
       <c r="B27" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15246</v>
+        <v>10000</v>
       </c>
       <c r="C27" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7736</v>
+        <v>20000</v>
       </c>
       <c r="D27" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>31927</v>
+        <v>30000</v>
       </c>
       <c r="E27" t="s">
         <v>244</v>
@@ -3885,16 +3739,13 @@
         <v>200</v>
       </c>
       <c r="B28" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>1611</v>
+        <v>10000</v>
       </c>
       <c r="C28" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>12891</v>
+        <v>20000</v>
       </c>
       <c r="D28" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>12660</v>
+        <v>30000</v>
       </c>
       <c r="E28" t="s">
         <v>244</v>
@@ -3908,16 +3759,13 @@
         <v>201</v>
       </c>
       <c r="B29" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32548</v>
+        <v>10000</v>
       </c>
       <c r="C29" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>514</v>
+        <v>20000</v>
       </c>
       <c r="D29" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39862</v>
+        <v>30000</v>
       </c>
       <c r="E29" t="s">
         <v>244</v>
@@ -3931,16 +3779,13 @@
         <v>202</v>
       </c>
       <c r="B30" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>621</v>
+        <v>10000</v>
       </c>
       <c r="C30" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>21440</v>
+        <v>20000</v>
       </c>
       <c r="D30" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>37076</v>
+        <v>30000</v>
       </c>
       <c r="E30" t="s">
         <v>244</v>
@@ -3954,16 +3799,13 @@
         <v>203</v>
       </c>
       <c r="B31" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>38179</v>
+        <v>10000</v>
       </c>
       <c r="C31" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39660</v>
+        <v>20000</v>
       </c>
       <c r="D31" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14996</v>
+        <v>30000</v>
       </c>
       <c r="E31" t="s">
         <v>244</v>
@@ -3977,16 +3819,13 @@
         <v>204</v>
       </c>
       <c r="B32" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>29919</v>
+        <v>10000</v>
       </c>
       <c r="C32" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>13207</v>
+        <v>20000</v>
       </c>
       <c r="D32" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3220</v>
+        <v>30000</v>
       </c>
       <c r="E32" t="s">
         <v>244</v>
@@ -4000,16 +3839,13 @@
         <v>205</v>
       </c>
       <c r="B33" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17168</v>
+        <v>10000</v>
       </c>
       <c r="C33" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>13900</v>
+        <v>20000</v>
       </c>
       <c r="D33" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>34892</v>
+        <v>30000</v>
       </c>
       <c r="E33" t="s">
         <v>244</v>
@@ -4023,16 +3859,13 @@
         <v>198</v>
       </c>
       <c r="B34" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>13690</v>
+        <v>10000</v>
       </c>
       <c r="C34" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>19973</v>
+        <v>20000</v>
       </c>
       <c r="D34" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>9825</v>
+        <v>30000</v>
       </c>
       <c r="E34" t="s">
         <v>244</v>
@@ -4046,16 +3879,13 @@
         <v>199</v>
       </c>
       <c r="B35" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>9850</v>
+        <v>10000</v>
       </c>
       <c r="C35" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>28125</v>
+        <v>20000</v>
       </c>
       <c r="D35" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>4560</v>
+        <v>30000</v>
       </c>
       <c r="E35" t="s">
         <v>244</v>
@@ -4069,16 +3899,13 @@
         <v>200</v>
       </c>
       <c r="B36" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8989</v>
+        <v>10000</v>
       </c>
       <c r="C36" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>1988</v>
+        <v>20000</v>
       </c>
       <c r="D36" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14601</v>
+        <v>30000</v>
       </c>
       <c r="E36" t="s">
         <v>244</v>
@@ -4092,16 +3919,13 @@
         <v>201</v>
       </c>
       <c r="B37" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27262</v>
+        <v>10000</v>
       </c>
       <c r="C37" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7827</v>
+        <v>20000</v>
       </c>
       <c r="D37" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8585</v>
+        <v>30000</v>
       </c>
       <c r="E37" t="s">
         <v>244</v>
@@ -4115,16 +3939,13 @@
         <v>202</v>
       </c>
       <c r="B38" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>23520</v>
+        <v>10000</v>
       </c>
       <c r="C38" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>24125</v>
+        <v>20000</v>
       </c>
       <c r="D38" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8882</v>
+        <v>30000</v>
       </c>
       <c r="E38" t="s">
         <v>244</v>
@@ -4138,16 +3959,13 @@
         <v>203</v>
       </c>
       <c r="B39" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>24173</v>
+        <v>10000</v>
       </c>
       <c r="C39" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7445</v>
+        <v>20000</v>
       </c>
       <c r="D39" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>29084</v>
+        <v>30000</v>
       </c>
       <c r="E39" t="s">
         <v>244</v>
@@ -4161,16 +3979,13 @@
         <v>204</v>
       </c>
       <c r="B40" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>31253</v>
+        <v>10000</v>
       </c>
       <c r="C40" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26584</v>
+        <v>20000</v>
       </c>
       <c r="D40" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>1850</v>
+        <v>30000</v>
       </c>
       <c r="E40" t="s">
         <v>244</v>
@@ -4184,16 +3999,13 @@
         <v>205</v>
       </c>
       <c r="B41" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36516</v>
+        <v>10000</v>
       </c>
       <c r="C41" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>5413</v>
+        <v>20000</v>
       </c>
       <c r="D41" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26517</v>
+        <v>30000</v>
       </c>
       <c r="E41" t="s">
         <v>244</v>
@@ -4207,16 +4019,13 @@
         <v>162</v>
       </c>
       <c r="B42" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15514</v>
+        <v>10000</v>
       </c>
       <c r="C42" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30967</v>
+        <v>20000</v>
       </c>
       <c r="D42" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>5348</v>
+        <v>30000</v>
       </c>
       <c r="E42" t="s">
         <v>244</v>
@@ -4230,16 +4039,13 @@
         <v>165</v>
       </c>
       <c r="B43" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>39048</v>
+        <v>10000</v>
       </c>
       <c r="C43" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17274</v>
+        <v>20000</v>
       </c>
       <c r="D43" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26359</v>
+        <v>30000</v>
       </c>
       <c r="E43" t="s">
         <v>244</v>
@@ -4253,16 +4059,13 @@
         <v>166</v>
       </c>
       <c r="B44" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17258</v>
+        <v>10000</v>
       </c>
       <c r="C44" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35781</v>
+        <v>20000</v>
       </c>
       <c r="D44" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>34808</v>
+        <v>30000</v>
       </c>
       <c r="E44" t="s">
         <v>244</v>
@@ -4276,16 +4079,13 @@
         <v>167</v>
       </c>
       <c r="B45" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36977</v>
+        <v>10000</v>
       </c>
       <c r="C45" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>10742</v>
+        <v>20000</v>
       </c>
       <c r="D45" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27120</v>
+        <v>30000</v>
       </c>
       <c r="E45" t="s">
         <v>244</v>
@@ -4299,16 +4099,13 @@
         <v>168</v>
       </c>
       <c r="B46" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3262</v>
+        <v>10000</v>
       </c>
       <c r="C46" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>18638</v>
+        <v>20000</v>
       </c>
       <c r="D46" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30311</v>
+        <v>30000</v>
       </c>
       <c r="E46" t="s">
         <v>244</v>
@@ -4322,16 +4119,13 @@
         <v>169</v>
       </c>
       <c r="B47" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>16977</v>
+        <v>10000</v>
       </c>
       <c r="C47" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>20532</v>
+        <v>20000</v>
       </c>
       <c r="D47" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>37310</v>
+        <v>30000</v>
       </c>
       <c r="E47" t="s">
         <v>244</v>
@@ -4345,16 +4139,13 @@
         <v>170</v>
       </c>
       <c r="B48" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>6998</v>
+        <v>10000</v>
       </c>
       <c r="C48" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35483</v>
+        <v>20000</v>
       </c>
       <c r="D48" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>10458</v>
+        <v>30000</v>
       </c>
       <c r="E48" t="s">
         <v>244</v>
@@ -4368,16 +4159,13 @@
         <v>171</v>
       </c>
       <c r="B49" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>20061</v>
+        <v>10000</v>
       </c>
       <c r="C49" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35237</v>
+        <v>20000</v>
       </c>
       <c r="D49" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>25710</v>
+        <v>30000</v>
       </c>
       <c r="E49" t="s">
         <v>244</v>
@@ -4391,16 +4179,13 @@
         <v>172</v>
       </c>
       <c r="B50" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>16421</v>
+        <v>10000</v>
       </c>
       <c r="C50" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>28499</v>
+        <v>20000</v>
       </c>
       <c r="D50" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17778</v>
+        <v>30000</v>
       </c>
       <c r="E50" t="s">
         <v>244</v>
@@ -4414,16 +4199,13 @@
         <v>173</v>
       </c>
       <c r="B51" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32486</v>
+        <v>10000</v>
       </c>
       <c r="C51" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30329</v>
+        <v>20000</v>
       </c>
       <c r="D51" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14871</v>
+        <v>30000</v>
       </c>
       <c r="E51" t="s">
         <v>244</v>
@@ -4437,16 +4219,13 @@
         <v>174</v>
       </c>
       <c r="B52" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>10909</v>
+        <v>10000</v>
       </c>
       <c r="C52" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>31966</v>
+        <v>20000</v>
       </c>
       <c r="D52" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>27287</v>
+        <v>30000</v>
       </c>
       <c r="E52" t="s">
         <v>244</v>
@@ -4460,16 +4239,13 @@
         <v>175</v>
       </c>
       <c r="B53" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>8978</v>
+        <v>10000</v>
       </c>
       <c r="C53" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35247</v>
+        <v>20000</v>
       </c>
       <c r="D53" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>26100</v>
+        <v>30000</v>
       </c>
       <c r="E53" t="s">
         <v>244</v>
@@ -4483,16 +4259,13 @@
         <v>176</v>
       </c>
       <c r="B54" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>12420</v>
+        <v>10000</v>
       </c>
       <c r="C54" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3860</v>
+        <v>20000</v>
       </c>
       <c r="D54" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>17506</v>
+        <v>30000</v>
       </c>
       <c r="E54" t="s">
         <v>244</v>
@@ -4506,16 +4279,13 @@
         <v>177</v>
       </c>
       <c r="B55" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>18306</v>
+        <v>10000</v>
       </c>
       <c r="C55" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>396</v>
+        <v>20000</v>
       </c>
       <c r="D55" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>23541</v>
+        <v>30000</v>
       </c>
       <c r="E55" t="s">
         <v>244</v>
@@ -4529,16 +4299,13 @@
         <v>162</v>
       </c>
       <c r="B56" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35206</v>
+        <v>10000</v>
       </c>
       <c r="C56" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>36119</v>
+        <v>20000</v>
       </c>
       <c r="D56" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>9068</v>
+        <v>30000</v>
       </c>
       <c r="E56" t="s">
         <v>244</v>
@@ -4552,16 +4319,13 @@
         <v>165</v>
       </c>
       <c r="B57" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30363</v>
+        <v>10000</v>
       </c>
       <c r="C57" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15492</v>
+        <v>20000</v>
       </c>
       <c r="D57" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7849</v>
+        <v>30000</v>
       </c>
       <c r="E57" t="s">
         <v>244</v>
@@ -4575,16 +4339,13 @@
         <v>166</v>
       </c>
       <c r="B58" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35516</v>
+        <v>10000</v>
       </c>
       <c r="C58" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>28275</v>
+        <v>20000</v>
       </c>
       <c r="D58" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7959</v>
+        <v>30000</v>
       </c>
       <c r="E58" t="s">
         <v>244</v>
@@ -4598,16 +4359,13 @@
         <v>167</v>
       </c>
       <c r="B59" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>2077</v>
+        <v>10000</v>
       </c>
       <c r="C59" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>33816</v>
+        <v>20000</v>
       </c>
       <c r="D59" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3093</v>
+        <v>30000</v>
       </c>
       <c r="E59" t="s">
         <v>244</v>
@@ -4621,16 +4379,13 @@
         <v>168</v>
       </c>
       <c r="B60" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>6186</v>
+        <v>10000</v>
       </c>
       <c r="C60" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>7968</v>
+        <v>20000</v>
       </c>
       <c r="D60" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>23202</v>
+        <v>30000</v>
       </c>
       <c r="E60" t="s">
         <v>244</v>
@@ -4644,16 +4399,13 @@
         <v>169</v>
       </c>
       <c r="B61" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>19525</v>
+        <v>10000</v>
       </c>
       <c r="C61" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>16004</v>
+        <v>20000</v>
       </c>
       <c r="D61" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35883</v>
+        <v>30000</v>
       </c>
       <c r="E61" t="s">
         <v>244</v>
@@ -4667,16 +4419,13 @@
         <v>170</v>
       </c>
       <c r="B62" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>14603</v>
+        <v>10000</v>
       </c>
       <c r="C62" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>25419</v>
+        <v>20000</v>
       </c>
       <c r="D62" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35878</v>
+        <v>30000</v>
       </c>
       <c r="E62" t="s">
         <v>244</v>
@@ -4690,16 +4439,13 @@
         <v>171</v>
       </c>
       <c r="B63" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>30668</v>
+        <v>10000</v>
       </c>
       <c r="C63" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>31413</v>
+        <v>20000</v>
       </c>
       <c r="D63" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>6697</v>
+        <v>30000</v>
       </c>
       <c r="E63" t="s">
         <v>244</v>
@@ -4713,16 +4459,13 @@
         <v>172</v>
       </c>
       <c r="B64" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>15489</v>
+        <v>10000</v>
       </c>
       <c r="C64" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>19131</v>
+        <v>20000</v>
       </c>
       <c r="D64" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>4191</v>
+        <v>30000</v>
       </c>
       <c r="E64" t="s">
         <v>244</v>
@@ -4736,16 +4479,13 @@
         <v>173</v>
       </c>
       <c r="B65" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>35641</v>
+        <v>10000</v>
       </c>
       <c r="C65" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>3114</v>
+        <v>20000</v>
       </c>
       <c r="D65" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>20188</v>
+        <v>30000</v>
       </c>
       <c r="E65" t="s">
         <v>244</v>
@@ -4759,16 +4499,13 @@
         <v>174</v>
       </c>
       <c r="B66" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>32425</v>
+        <v>10000</v>
       </c>
       <c r="C66" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>24847</v>
+        <v>20000</v>
       </c>
       <c r="D66" s="3">
-        <f t="shared" ca="1" si="0"/>
-        <v>24852</v>
+        <v>30000</v>
       </c>
       <c r="E66" t="s">
         <v>244</v>
@@ -4782,16 +4519,13 @@
         <v>175</v>
       </c>
       <c r="B67" s="3">
-        <f t="shared" ref="B67:D69" ca="1" si="1">RANDBETWEEN(0,40000)</f>
-        <v>34019</v>
+        <v>10000</v>
       </c>
       <c r="C67" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>25403</v>
+        <v>20000</v>
       </c>
       <c r="D67" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>4245</v>
+        <v>30000</v>
       </c>
       <c r="E67" t="s">
         <v>244</v>
@@ -4805,16 +4539,13 @@
         <v>176</v>
       </c>
       <c r="B68" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>11174</v>
+        <v>10000</v>
       </c>
       <c r="C68" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>33622</v>
+        <v>20000</v>
       </c>
       <c r="D68" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>23994</v>
+        <v>30000</v>
       </c>
       <c r="E68" t="s">
         <v>244</v>
@@ -4828,16 +4559,13 @@
         <v>177</v>
       </c>
       <c r="B69" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>378</v>
+        <v>10000</v>
       </c>
       <c r="C69" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>39242</v>
+        <v>20000</v>
       </c>
       <c r="D69" s="3">
-        <f t="shared" ca="1" si="1"/>
-        <v>1549</v>
+        <v>30000</v>
       </c>
       <c r="E69" t="s">
         <v>244</v>
@@ -4885,16 +4613,13 @@
         <v>191</v>
       </c>
       <c r="B2" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>240</v>
+        <v>100</v>
       </c>
       <c r="C2" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>47</v>
+        <v>150</v>
       </c>
       <c r="D2" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="E2" t="s">
         <v>244</v>
@@ -4905,16 +4630,13 @@
         <v>192</v>
       </c>
       <c r="B3" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="C3" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="D3" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>260</v>
+        <v>200</v>
       </c>
       <c r="E3" t="s">
         <v>244</v>
@@ -4925,16 +4647,13 @@
         <v>206</v>
       </c>
       <c r="B4" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>36</v>
+        <v>100</v>
       </c>
       <c r="C4" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>4</v>
+        <v>150</v>
       </c>
       <c r="D4" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>290</v>
+        <v>200</v>
       </c>
       <c r="E4" t="s">
         <v>244</v>
@@ -4945,16 +4664,13 @@
         <v>193</v>
       </c>
       <c r="B5" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="C5" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>229</v>
+        <v>150</v>
       </c>
       <c r="D5" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>257</v>
+        <v>200</v>
       </c>
       <c r="E5" t="s">
         <v>244</v>
@@ -4965,16 +4681,13 @@
         <v>140</v>
       </c>
       <c r="B6" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>213</v>
+        <v>100</v>
       </c>
       <c r="C6" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>17</v>
+        <v>150</v>
       </c>
       <c r="D6" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>263</v>
+        <v>200</v>
       </c>
       <c r="E6" t="s">
         <v>226</v>
@@ -4985,16 +4698,13 @@
         <v>153</v>
       </c>
       <c r="B7" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>265</v>
+        <v>100</v>
       </c>
       <c r="C7" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="D7" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E7" t="s">
         <v>244</v>
@@ -5005,16 +4715,13 @@
         <v>141</v>
       </c>
       <c r="B8" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>223</v>
+        <v>100</v>
       </c>
       <c r="C8" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="D8" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="E8" t="s">
         <v>226</v>
@@ -5025,16 +4732,13 @@
         <v>194</v>
       </c>
       <c r="B9" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="C9" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>199</v>
+        <v>150</v>
       </c>
       <c r="D9" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>92</v>
+        <v>200</v>
       </c>
       <c r="E9" t="s">
         <v>244</v>
@@ -5045,16 +4749,13 @@
         <v>207</v>
       </c>
       <c r="B10" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>149</v>
+        <v>100</v>
       </c>
       <c r="C10" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D10" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>269</v>
+        <v>200</v>
       </c>
       <c r="E10" t="s">
         <v>244</v>
@@ -5065,16 +4766,13 @@
         <v>208</v>
       </c>
       <c r="B11" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>268</v>
+        <v>100</v>
       </c>
       <c r="C11" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>219</v>
+        <v>150</v>
       </c>
       <c r="D11" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>69</v>
+        <v>200</v>
       </c>
       <c r="E11" t="s">
         <v>244</v>
@@ -5085,16 +4783,13 @@
         <v>154</v>
       </c>
       <c r="B12" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>299</v>
+        <v>100</v>
       </c>
       <c r="C12" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>78</v>
+        <v>150</v>
       </c>
       <c r="D12" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>116</v>
+        <v>200</v>
       </c>
       <c r="E12" t="s">
         <v>244</v>
@@ -5105,16 +4800,13 @@
         <v>178</v>
       </c>
       <c r="B13" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C13" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="D13" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>258</v>
+        <v>200</v>
       </c>
       <c r="E13" t="s">
         <v>244</v>
@@ -5125,16 +4817,13 @@
         <v>209</v>
       </c>
       <c r="B14" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="C14" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D14" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>119</v>
+        <v>200</v>
       </c>
       <c r="E14" t="s">
         <v>244</v>
@@ -5145,16 +4834,13 @@
         <v>142</v>
       </c>
       <c r="B15" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>172</v>
+        <v>100</v>
       </c>
       <c r="C15" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="D15" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>142</v>
+        <v>200</v>
       </c>
       <c r="E15" t="s">
         <v>226</v>
@@ -5165,16 +4851,13 @@
         <v>143</v>
       </c>
       <c r="B16" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>277</v>
+        <v>100</v>
       </c>
       <c r="C16" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="D16" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>258</v>
+        <v>200</v>
       </c>
       <c r="E16" t="s">
         <v>226</v>
@@ -5185,16 +4868,13 @@
         <v>155</v>
       </c>
       <c r="B17" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>225</v>
+        <v>100</v>
       </c>
       <c r="C17" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="D17" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>276</v>
+        <v>200</v>
       </c>
       <c r="E17" t="s">
         <v>244</v>
@@ -5205,16 +4885,13 @@
         <v>156</v>
       </c>
       <c r="B18" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="C18" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>295</v>
+        <v>150</v>
       </c>
       <c r="D18" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>247</v>
+        <v>200</v>
       </c>
       <c r="E18" t="s">
         <v>244</v>
@@ -5225,16 +4902,13 @@
         <v>157</v>
       </c>
       <c r="B19" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="C19" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>52</v>
+        <v>150</v>
       </c>
       <c r="D19" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="E19" t="s">
         <v>244</v>
@@ -5245,16 +4919,13 @@
         <v>130</v>
       </c>
       <c r="B20" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="C20" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>102</v>
+        <v>150</v>
       </c>
       <c r="D20" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>152</v>
+        <v>200</v>
       </c>
       <c r="E20" t="s">
         <v>225</v>
@@ -5265,16 +4936,13 @@
         <v>131</v>
       </c>
       <c r="B21" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C21" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="D21" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>293</v>
+        <v>200</v>
       </c>
       <c r="E21" t="s">
         <v>225</v>
@@ -5285,16 +4953,13 @@
         <v>158</v>
       </c>
       <c r="B22" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="C22" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>56</v>
+        <v>150</v>
       </c>
       <c r="D22" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>166</v>
+        <v>200</v>
       </c>
       <c r="E22" t="s">
         <v>244</v>
@@ -5305,16 +4970,13 @@
         <v>210</v>
       </c>
       <c r="B23" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>211</v>
+        <v>100</v>
       </c>
       <c r="C23" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>189</v>
+        <v>150</v>
       </c>
       <c r="D23" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>79</v>
+        <v>200</v>
       </c>
       <c r="E23" t="s">
         <v>244</v>
@@ -5325,16 +4987,13 @@
         <v>179</v>
       </c>
       <c r="B24" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="C24" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>68</v>
+        <v>150</v>
       </c>
       <c r="D24" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>23</v>
+        <v>200</v>
       </c>
       <c r="E24" t="s">
         <v>244</v>
@@ -5345,16 +5004,13 @@
         <v>180</v>
       </c>
       <c r="B25" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>237</v>
+        <v>100</v>
       </c>
       <c r="C25" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>259</v>
+        <v>150</v>
       </c>
       <c r="D25" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E25" t="s">
         <v>244</v>
@@ -5365,16 +5021,13 @@
         <v>181</v>
       </c>
       <c r="B26" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="C26" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D26" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>69</v>
+        <v>200</v>
       </c>
       <c r="E26" t="s">
         <v>244</v>
@@ -5385,16 +5038,13 @@
         <v>182</v>
       </c>
       <c r="B27" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="C27" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>294</v>
+        <v>150</v>
       </c>
       <c r="D27" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>4</v>
+        <v>200</v>
       </c>
       <c r="E27" t="s">
         <v>244</v>
@@ -5405,16 +5055,13 @@
         <v>183</v>
       </c>
       <c r="B28" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="C28" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="D28" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>182</v>
+        <v>200</v>
       </c>
       <c r="E28" t="s">
         <v>244</v>
@@ -5425,16 +5072,13 @@
         <v>132</v>
       </c>
       <c r="B29" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C29" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>28</v>
+        <v>150</v>
       </c>
       <c r="D29" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>117</v>
+        <v>200</v>
       </c>
       <c r="E29" t="s">
         <v>225</v>
@@ -5445,16 +5089,13 @@
         <v>133</v>
       </c>
       <c r="B30" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>244</v>
+        <v>100</v>
       </c>
       <c r="C30" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>7</v>
+        <v>150</v>
       </c>
       <c r="D30" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>14</v>
+        <v>200</v>
       </c>
       <c r="E30" t="s">
         <v>225</v>
@@ -5465,16 +5106,13 @@
         <v>195</v>
       </c>
       <c r="B31" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="C31" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>286</v>
+        <v>150</v>
       </c>
       <c r="D31" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>17</v>
+        <v>200</v>
       </c>
       <c r="E31" t="s">
         <v>244</v>
@@ -5485,16 +5123,13 @@
         <v>211</v>
       </c>
       <c r="B32" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>52</v>
+        <v>100</v>
       </c>
       <c r="C32" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="D32" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="E32" t="s">
         <v>244</v>
@@ -5505,16 +5140,13 @@
         <v>212</v>
       </c>
       <c r="B33" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="C33" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>223</v>
+        <v>150</v>
       </c>
       <c r="D33" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>261</v>
+        <v>200</v>
       </c>
       <c r="E33" t="s">
         <v>244</v>
@@ -5525,16 +5157,13 @@
         <v>196</v>
       </c>
       <c r="B34" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="C34" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="D34" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="E34" t="s">
         <v>244</v>
@@ -5545,16 +5174,13 @@
         <v>197</v>
       </c>
       <c r="B35" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="C35" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D35" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E35" t="s">
         <v>244</v>
@@ -5565,16 +5191,13 @@
         <v>159</v>
       </c>
       <c r="B36" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>251</v>
+        <v>100</v>
       </c>
       <c r="C36" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>231</v>
+        <v>150</v>
       </c>
       <c r="D36" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="E36" t="s">
         <v>244</v>
@@ -5585,16 +5208,13 @@
         <v>213</v>
       </c>
       <c r="B37" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="C37" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>235</v>
+        <v>150</v>
       </c>
       <c r="D37" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="E37" t="s">
         <v>244</v>
@@ -5605,16 +5225,13 @@
         <v>160</v>
       </c>
       <c r="B38" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="C38" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>194</v>
+        <v>150</v>
       </c>
       <c r="D38" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>137</v>
+        <v>200</v>
       </c>
       <c r="E38" t="s">
         <v>244</v>
@@ -5625,16 +5242,13 @@
         <v>144</v>
       </c>
       <c r="B39" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>194</v>
+        <v>100</v>
       </c>
       <c r="C39" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="D39" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>148</v>
+        <v>200</v>
       </c>
       <c r="E39" t="s">
         <v>226</v>
@@ -5645,16 +5259,13 @@
         <v>145</v>
       </c>
       <c r="B40" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>243</v>
+        <v>100</v>
       </c>
       <c r="C40" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>214</v>
+        <v>150</v>
       </c>
       <c r="D40" s="3">
-        <f ca="1">RANDBETWEEN(0,300)</f>
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E40" t="s">
         <v>226</v>

</xml_diff>